<commit_message>
feat: standardise schedule cell color status matrix (white, green, blue, orange, red) and connect to dashboard
</commit_message>
<xml_diff>
--- a/file_wisuda_3okt.xlsx
+++ b/file_wisuda_3okt.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="81">
   <si>
     <t xml:space="preserve">Graduation Schedule 
 </t>
@@ -103,147 +103,144 @@
     <t>AD</t>
   </si>
   <si>
+    <t xml:space="preserve"> Fadila</t>
+  </si>
+  <si>
+    <t>Rani</t>
+  </si>
+  <si>
+    <t>Qotrunnada Maulidia</t>
+  </si>
+  <si>
+    <t>Nasywaa</t>
+  </si>
+  <si>
+    <t>Mufti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Graduation </t>
+  </si>
+  <si>
+    <t>Ilut</t>
+  </si>
+  <si>
+    <t>nabila hasna</t>
+  </si>
+  <si>
+    <t>Logi</t>
+  </si>
+  <si>
+    <t>Aulia Hani</t>
+  </si>
+  <si>
+    <t>Windi</t>
+  </si>
+  <si>
+    <t>Shabrina Amalia</t>
+  </si>
+  <si>
+    <t>Nana</t>
+  </si>
+  <si>
+    <t>Wafi Wafa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Tika Dwi</t>
+  </si>
+  <si>
+    <t>Devinta Khoerunnisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> oktriana</t>
+  </si>
+  <si>
+    <t>N. A. Salsabila</t>
+  </si>
+  <si>
+    <t>Rahayu Purnama</t>
+  </si>
+  <si>
+    <t>Graduatiom</t>
+  </si>
+  <si>
+    <t>Gandring Guste Puand</t>
+  </si>
+  <si>
+    <t>Graduatio prem</t>
+  </si>
+  <si>
+    <t>Afifah</t>
+  </si>
+  <si>
+    <t>Zaidan Ariefyandi</t>
+  </si>
+  <si>
+    <t>Sandlyra Anastasya</t>
+  </si>
+  <si>
+    <t>helmi</t>
+  </si>
+  <si>
+    <t>Reynaldo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> widyaloka</t>
+  </si>
+  <si>
+    <t>Amelia Nur</t>
+  </si>
+  <si>
+    <t>calresta</t>
+  </si>
+  <si>
+    <t>Niko</t>
+  </si>
+  <si>
+    <t>Wahyu Setianingsih</t>
+  </si>
+  <si>
+    <t>Karlina</t>
+  </si>
+  <si>
+    <t>Nabilla</t>
+  </si>
+  <si>
+    <t>Tiffani Agil</t>
+  </si>
+  <si>
+    <t>Nina Dwi Suryani</t>
+  </si>
+  <si>
+    <t>Mahendra Putra Wardhana</t>
+  </si>
+  <si>
+    <t>Afita Khoerunnisa</t>
+  </si>
+  <si>
+    <t>Dita</t>
+  </si>
+  <si>
+    <t>Sifa</t>
+  </si>
+  <si>
+    <t>Hanifa</t>
+  </si>
+  <si>
+    <t>Akhmad binangun</t>
+  </si>
+  <si>
+    <t>lala</t>
+  </si>
+  <si>
+    <t>sabrina</t>
+  </si>
+  <si>
     <t>Claresta</t>
   </si>
   <si>
-    <t xml:space="preserve">Graduation </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Fadila</t>
-  </si>
-  <si>
-    <t>Rani</t>
-  </si>
-  <si>
-    <t>Rahayu Purnama</t>
-  </si>
-  <si>
-    <t>Graduatiom</t>
-  </si>
-  <si>
-    <t>Qotrunnada Maulidia</t>
-  </si>
-  <si>
-    <t>Nasywaa</t>
-  </si>
-  <si>
-    <t>Mufti</t>
-  </si>
-  <si>
-    <t>Ilut</t>
-  </si>
-  <si>
-    <t>nabila hasna</t>
-  </si>
-  <si>
-    <t>Logi</t>
-  </si>
-  <si>
-    <t>Aulia Hani</t>
-  </si>
-  <si>
-    <t>Windi</t>
-  </si>
-  <si>
-    <t>Shabrina Amalia</t>
-  </si>
-  <si>
-    <t>Nana</t>
-  </si>
-  <si>
-    <t>Wafi Wafa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Tika Dwi</t>
-  </si>
-  <si>
-    <t>Devinta Khoerunnisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> oktriana</t>
-  </si>
-  <si>
-    <t>N. A. Salsabila</t>
-  </si>
-  <si>
-    <t>Gandring Guste Puand</t>
-  </si>
-  <si>
-    <t>Graduatio prem</t>
-  </si>
-  <si>
-    <t>Afifah</t>
-  </si>
-  <si>
-    <t>Zaidan Ariefyandi</t>
-  </si>
-  <si>
-    <t>Sandlyra Anastasya</t>
-  </si>
-  <si>
-    <t>helmi</t>
-  </si>
-  <si>
-    <t>Reynaldo</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> widyaloka</t>
-  </si>
-  <si>
-    <t>Amelia Nur</t>
-  </si>
-  <si>
-    <t>Syifa Zulfa</t>
-  </si>
-  <si>
-    <t>Niko</t>
-  </si>
-  <si>
-    <t>Wahyu Setianingsih</t>
-  </si>
-  <si>
-    <t>Karlina</t>
-  </si>
-  <si>
-    <t>Nabilla</t>
-  </si>
-  <si>
-    <t>Tiffani Agil</t>
-  </si>
-  <si>
-    <t>Nina Dwi Suryani</t>
-  </si>
-  <si>
-    <t>Mahendra Putra Wardhana</t>
-  </si>
-  <si>
-    <t>Afita Khoerunnisa</t>
-  </si>
-  <si>
     <t>CLOSED</t>
   </si>
   <si>
-    <t>Dita</t>
-  </si>
-  <si>
-    <t>Sifa</t>
-  </si>
-  <si>
-    <t>Hanifa</t>
-  </si>
-  <si>
-    <t>Akhmad binangun</t>
-  </si>
-  <si>
-    <t>lala</t>
-  </si>
-  <si>
-    <t>sabrina</t>
-  </si>
-  <si>
-    <t>Cahya Juwita</t>
-  </si>
-  <si>
     <t>Desti Ika c</t>
   </si>
   <si>
@@ -257,6 +254,9 @@
   </si>
   <si>
     <t>Graaduation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indah </t>
   </si>
   <si>
     <t xml:space="preserve"> Uji</t>
@@ -411,14 +411,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF9900"/>
-        <bgColor rgb="FFFF9900"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF0000"/>
+        <fgColor rgb="FFFF9900"/>
+        <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
     <fill>
@@ -428,7 +428,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border/>
     <border>
       <right style="thin">
@@ -535,6 +535,11 @@
       </bottom>
     </border>
     <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+    </border>
+    <border>
       <top style="dotted">
         <color rgb="FF000000"/>
       </top>
@@ -590,7 +595,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="84">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -680,125 +685,155 @@
     <xf borderId="6" fillId="9" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="15" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="8" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="8" fillId="9" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="10" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="12" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="10" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="10" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="12" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="5" fillId="12" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="8" fillId="12" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="9" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="5" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="5" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="10" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="12" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="8" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="12" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="12" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="5" fillId="12" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="8" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="13" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="13" fillId="0" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="13" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="13" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="13" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="14" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="15" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="12" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="13" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -821,7 +856,7 @@
     <xdr:ext cx="2590800" cy="2590800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Gambar"/>
+        <xdr:cNvPr id="0" name="image6.png" title="Gambar"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -877,7 +912,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.jpg"/>
+        <xdr:cNvPr id="0" name="image3.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -905,7 +940,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.jpg"/>
+        <xdr:cNvPr id="0" name="image5.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -933,7 +968,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.jpg"/>
+        <xdr:cNvPr id="0" name="image2.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -961,7 +996,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.jpg"/>
+        <xdr:cNvPr id="0" name="image4.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1835,10 +1870,10 @@
       <c r="P19" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="Q19" s="31" t="s">
+      <c r="Q19" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="R19" s="31" t="s">
+      <c r="R19" s="25" t="s">
         <v>16</v>
       </c>
       <c r="S19" s="21">
@@ -1847,66 +1882,66 @@
       <c r="T19" s="22">
         <v>0.5208333333333334</v>
       </c>
-      <c r="U19" s="32"/>
-      <c r="V19" s="32"/>
-      <c r="W19" s="32"/>
-      <c r="X19" s="32"/>
-      <c r="Y19" s="33">
+      <c r="U19" s="31"/>
+      <c r="V19" s="31"/>
+      <c r="W19" s="31"/>
+      <c r="X19" s="31"/>
+      <c r="Y19" s="32">
         <v>8.0</v>
       </c>
-      <c r="Z19" s="34">
+      <c r="Z19" s="33">
         <v>0.5208333333333334</v>
       </c>
-      <c r="AA19" s="35"/>
-      <c r="AB19" s="35"/>
-      <c r="AC19" s="35"/>
-      <c r="AD19" s="35"/>
+      <c r="AA19" s="34"/>
+      <c r="AB19" s="34"/>
+      <c r="AC19" s="34"/>
+      <c r="AD19" s="34"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="36">
+      <c r="A20" s="35">
         <v>9.0</v>
       </c>
-      <c r="B20" s="37">
+      <c r="B20" s="36">
         <v>0.5416666666666666</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="D20" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="38" t="s">
+      <c r="D20" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="F20" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="39">
+      <c r="F20" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="38">
         <v>9.0</v>
       </c>
-      <c r="H20" s="40">
+      <c r="H20" s="39">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="39"/>
-      <c r="M20" s="41">
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
+      <c r="K20" s="34"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="35">
         <v>9.0</v>
       </c>
-      <c r="N20" s="42">
+      <c r="N20" s="36">
         <v>0.5416666666666666</v>
       </c>
-      <c r="O20" s="43" t="s">
+      <c r="O20" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="P20" s="44" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q20" s="44" t="s">
+      <c r="P20" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q20" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="R20" s="44" t="s">
+      <c r="R20" s="41" t="s">
         <v>16</v>
       </c>
       <c r="S20" s="23">
@@ -1915,16 +1950,16 @@
       <c r="T20" s="24">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U20" s="38" t="s">
+      <c r="U20" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="V20" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="W20" s="38" t="s">
+      <c r="V20" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="W20" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="X20" s="38" t="s">
+      <c r="X20" s="25" t="s">
         <v>16</v>
       </c>
       <c r="Y20" s="23">
@@ -1942,63 +1977,55 @@
       <c r="AC20" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="AD20" s="38" t="s">
+      <c r="AD20" s="25" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="45">
+      <c r="A21" s="42">
         <v>10.0</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="43">
         <v>0.5555555555555556</v>
       </c>
-      <c r="C21" s="45" t="s">
+      <c r="C21" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="45" t="s">
+      <c r="D21" s="42" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="F21" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="36">
+      <c r="F21" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="38">
         <v>10.0</v>
       </c>
-      <c r="H21" s="37">
+      <c r="H21" s="39">
         <v>0.5555555555555556</v>
       </c>
-      <c r="I21" s="45" t="s">
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="44"/>
+      <c r="M21" s="35">
+        <v>10.0</v>
+      </c>
+      <c r="N21" s="45">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="O21" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="J21" s="45" t="s">
-        <v>29</v>
-      </c>
-      <c r="K21" s="45" t="s">
-        <v>15</v>
-      </c>
-      <c r="L21" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="M21" s="36">
-        <v>10.0</v>
-      </c>
-      <c r="N21" s="47">
-        <v>0.5555555555555556</v>
-      </c>
-      <c r="O21" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="P21" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q21" s="38" t="s">
+      <c r="P21" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q21" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="R21" s="38" t="s">
+      <c r="R21" s="37" t="s">
         <v>16</v>
       </c>
       <c r="S21" s="23">
@@ -2007,994 +2034,1022 @@
       <c r="T21" s="24">
         <v>0.5555555555555556</v>
       </c>
-      <c r="U21" s="50" t="s">
-        <v>31</v>
-      </c>
-      <c r="V21" s="50" t="s">
-        <v>14</v>
-      </c>
-      <c r="W21" s="50" t="s">
+      <c r="U21" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="V21" s="48" t="s">
+        <v>14</v>
+      </c>
+      <c r="W21" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="X21" s="51" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y21" s="39">
+      <c r="X21" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y21" s="38">
         <v>10.0</v>
       </c>
-      <c r="Z21" s="40">
+      <c r="Z21" s="39">
         <v>0.5555555555555556</v>
       </c>
-      <c r="AA21" s="39"/>
-      <c r="AB21" s="39"/>
-      <c r="AC21" s="39"/>
-      <c r="AD21" s="39"/>
+      <c r="AA21" s="38"/>
+      <c r="AB21" s="38"/>
+      <c r="AC21" s="38"/>
+      <c r="AD21" s="38"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="36">
+      <c r="A22" s="21">
         <v>11.0</v>
       </c>
-      <c r="B22" s="37">
+      <c r="B22" s="22">
         <v>0.5694444444444444</v>
       </c>
-      <c r="C22" s="38" t="s">
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="23">
+        <v>11.0</v>
+      </c>
+      <c r="H22" s="24">
+        <v>0.5694444444444444</v>
+      </c>
+      <c r="I22" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="J22" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="K22" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="L22" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="M22" s="23">
+        <v>11.0</v>
+      </c>
+      <c r="N22" s="50">
+        <v>0.5694444444444444</v>
+      </c>
+      <c r="O22" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="P22" s="52" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q22" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="R22" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="S22" s="38">
+        <v>11.0</v>
+      </c>
+      <c r="T22" s="39">
+        <v>0.5694444444444444</v>
+      </c>
+      <c r="U22" s="34"/>
+      <c r="V22" s="34"/>
+      <c r="W22" s="34"/>
+      <c r="X22" s="34"/>
+      <c r="Y22" s="23">
+        <v>11.0</v>
+      </c>
+      <c r="Z22" s="24">
+        <v>0.5694444444444444</v>
+      </c>
+      <c r="AA22" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="AB22" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="38" t="s">
+      <c r="AC22" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="F22" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G22" s="36">
-        <v>11.0</v>
-      </c>
-      <c r="H22" s="37">
-        <v>0.5694444444444444</v>
-      </c>
-      <c r="I22" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="J22" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K22" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="L22" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M22" s="36">
-        <v>11.0</v>
-      </c>
-      <c r="N22" s="47">
-        <v>0.5694444444444444</v>
-      </c>
-      <c r="O22" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="P22" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q22" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="R22" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S22" s="39">
-        <v>11.0</v>
-      </c>
-      <c r="T22" s="40">
-        <v>0.5694444444444444</v>
-      </c>
-      <c r="U22" s="35"/>
-      <c r="V22" s="35"/>
-      <c r="W22" s="35"/>
-      <c r="X22" s="35"/>
-      <c r="Y22" s="36">
-        <v>11.0</v>
-      </c>
-      <c r="Z22" s="37">
-        <v>0.5694444444444444</v>
-      </c>
-      <c r="AA22" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="AB22" s="38" t="s">
-        <v>29</v>
-      </c>
-      <c r="AC22" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="AD22" s="38" t="s">
+      <c r="AD22" s="25" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="36">
+      <c r="A23" s="23">
         <v>12.0</v>
       </c>
-      <c r="B23" s="37">
+      <c r="B23" s="24">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C23" s="38" t="s">
+      <c r="C23" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="23">
+        <v>12.0</v>
+      </c>
+      <c r="H23" s="24">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="I23" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="J23" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="K23" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="L23" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="M23" s="35">
+        <v>12.0</v>
+      </c>
+      <c r="N23" s="45">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="O23" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="P23" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q23" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="R23" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="S23" s="35">
+        <v>12.0</v>
+      </c>
+      <c r="T23" s="36">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="U23" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="36">
+      <c r="V23" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="W23" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="X23" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y23" s="38">
         <v>12.0</v>
       </c>
-      <c r="H23" s="37">
+      <c r="Z23" s="39">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I23" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="J23" s="52" t="s">
-        <v>14</v>
-      </c>
-      <c r="K23" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="L23" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M23" s="36">
-        <v>12.0</v>
-      </c>
-      <c r="N23" s="47">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="O23" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="P23" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q23" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="R23" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S23" s="36">
-        <v>12.0</v>
-      </c>
-      <c r="T23" s="37">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="U23" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="V23" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="W23" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="X23" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y23" s="39">
-        <v>12.0</v>
-      </c>
-      <c r="Z23" s="40">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="AA23" s="39"/>
-      <c r="AB23" s="39"/>
-      <c r="AC23" s="39"/>
-      <c r="AD23" s="39"/>
+      <c r="AA23" s="38"/>
+      <c r="AB23" s="38"/>
+      <c r="AC23" s="38"/>
+      <c r="AD23" s="38"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="36">
+      <c r="A24" s="35">
         <v>13.0</v>
       </c>
-      <c r="B24" s="37">
+      <c r="B24" s="36">
         <v>0.5972222222222222</v>
       </c>
-      <c r="C24" s="38" t="s">
+      <c r="C24" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="35">
+        <v>13.0</v>
+      </c>
+      <c r="H24" s="36">
+        <v>0.5972222222222222</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="L24" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="M24" s="35">
+        <v>13.0</v>
+      </c>
+      <c r="N24" s="36">
+        <v>0.5972222222222222</v>
+      </c>
+      <c r="O24" s="56" t="s">
+        <v>40</v>
+      </c>
+      <c r="P24" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q24" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="R24" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="S24" s="23">
+        <v>13.0</v>
+      </c>
+      <c r="T24" s="24">
+        <v>0.5972222222222222</v>
+      </c>
+      <c r="U24" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G24" s="36">
+      <c r="V24" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="W24" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="X24" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y24" s="38">
         <v>13.0</v>
       </c>
-      <c r="H24" s="37">
+      <c r="Z24" s="39">
         <v>0.5972222222222222</v>
       </c>
-      <c r="I24" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="J24" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K24" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="L24" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M24" s="36">
-        <v>13.0</v>
-      </c>
-      <c r="N24" s="37">
-        <v>0.5972222222222222</v>
-      </c>
-      <c r="O24" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="P24" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q24" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="R24" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S24" s="36">
-        <v>13.0</v>
-      </c>
-      <c r="T24" s="37">
-        <v>0.5972222222222222</v>
-      </c>
-      <c r="U24" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="V24" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="W24" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="X24" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y24" s="39">
-        <v>13.0</v>
-      </c>
-      <c r="Z24" s="40">
-        <v>0.5972222222222222</v>
-      </c>
-      <c r="AA24" s="39"/>
-      <c r="AB24" s="39"/>
-      <c r="AC24" s="39"/>
-      <c r="AD24" s="39"/>
+      <c r="AA24" s="38"/>
+      <c r="AB24" s="38"/>
+      <c r="AC24" s="38"/>
+      <c r="AD24" s="38"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="36">
+      <c r="A25" s="57">
         <v>14.0</v>
       </c>
-      <c r="B25" s="37">
+      <c r="B25" s="58">
         <v>0.6111111111111112</v>
       </c>
-      <c r="C25" s="38" t="s">
+      <c r="C25" s="53" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="57">
+        <v>14.0</v>
+      </c>
+      <c r="H25" s="58">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="I25" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="J25" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K25" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="L25" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M25" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="N25" s="24">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="O25" s="53" t="s">
+        <v>44</v>
+      </c>
+      <c r="P25" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q25" s="53" t="s">
+        <v>27</v>
+      </c>
+      <c r="R25" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="S25" s="38">
+        <v>14.0</v>
+      </c>
+      <c r="T25" s="39">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="U25" s="38"/>
+      <c r="V25" s="38"/>
+      <c r="W25" s="38"/>
+      <c r="X25" s="38"/>
+      <c r="Y25" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="Z25" s="24">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="AA25" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="D25" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G25" s="36">
-        <v>14.0</v>
-      </c>
-      <c r="H25" s="37">
-        <v>0.6111111111111112</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="J25" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K25" s="38" t="s">
+      <c r="AB25" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC25" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="L25" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M25" s="36">
-        <v>14.0</v>
-      </c>
-      <c r="N25" s="37">
-        <v>0.6111111111111112</v>
-      </c>
-      <c r="O25" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="P25" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q25" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="R25" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S25" s="39">
-        <v>14.0</v>
-      </c>
-      <c r="T25" s="40">
-        <v>0.6111111111111112</v>
-      </c>
-      <c r="U25" s="39"/>
-      <c r="V25" s="39"/>
-      <c r="W25" s="39"/>
-      <c r="X25" s="39"/>
-      <c r="Y25" s="36">
-        <v>14.0</v>
-      </c>
-      <c r="Z25" s="37">
-        <v>0.6111111111111112</v>
-      </c>
-      <c r="AA25" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB25" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC25" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="AD25" s="38" t="s">
+      <c r="AD25" s="53" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="36">
+      <c r="A26" s="23">
         <v>15.0</v>
       </c>
-      <c r="B26" s="37">
+      <c r="B26" s="24">
         <v>0.625</v>
       </c>
-      <c r="C26" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E26" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G26" s="36">
+      <c r="C26" s="53" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="53" t="s">
+        <v>47</v>
+      </c>
+      <c r="E26" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="57">
         <v>15.0</v>
       </c>
-      <c r="H26" s="37">
+      <c r="H26" s="58">
         <v>0.625</v>
       </c>
-      <c r="I26" s="38" t="s">
+      <c r="I26" s="53" t="s">
+        <v>48</v>
+      </c>
+      <c r="J26" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="J26" s="38" t="s">
+      <c r="K26" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="L26" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M26" s="57">
+        <v>15.0</v>
+      </c>
+      <c r="N26" s="58">
+        <v>0.625</v>
+      </c>
+      <c r="O26" s="57" t="s">
         <v>50</v>
       </c>
-      <c r="K26" s="38" t="s">
+      <c r="P26" s="57" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q26" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="R26" s="59" t="s">
+        <v>16</v>
+      </c>
+      <c r="S26" s="38">
+        <v>15.0</v>
+      </c>
+      <c r="T26" s="39">
+        <v>0.625</v>
+      </c>
+      <c r="U26" s="38"/>
+      <c r="V26" s="38"/>
+      <c r="W26" s="38"/>
+      <c r="X26" s="38"/>
+      <c r="Y26" s="57">
+        <v>15.0</v>
+      </c>
+      <c r="Z26" s="58">
+        <v>0.625</v>
+      </c>
+      <c r="AA26" s="53" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB26" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC26" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="L26" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M26" s="36">
-        <v>15.0</v>
-      </c>
-      <c r="N26" s="37">
-        <v>0.625</v>
-      </c>
-      <c r="O26" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="P26" s="36" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q26" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="R26" s="48" t="s">
-        <v>16</v>
-      </c>
-      <c r="S26" s="39">
-        <v>15.0</v>
-      </c>
-      <c r="T26" s="40">
-        <v>0.625</v>
-      </c>
-      <c r="U26" s="39"/>
-      <c r="V26" s="39"/>
-      <c r="W26" s="39"/>
-      <c r="X26" s="39"/>
-      <c r="Y26" s="36">
-        <v>15.0</v>
-      </c>
-      <c r="Z26" s="37">
-        <v>0.625</v>
-      </c>
-      <c r="AA26" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB26" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC26" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="AD26" s="38" t="s">
+      <c r="AD26" s="53" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="36">
+      <c r="A27" s="57">
         <v>16.0</v>
       </c>
-      <c r="B27" s="37">
+      <c r="B27" s="58">
         <v>0.6388888888888888</v>
       </c>
-      <c r="C27" s="38" t="s">
+      <c r="C27" s="53" t="s">
+        <v>52</v>
+      </c>
+      <c r="D27" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="57">
+        <v>16.0</v>
+      </c>
+      <c r="H27" s="58">
+        <v>0.6388888888888888</v>
+      </c>
+      <c r="I27" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="38" t="s">
+      <c r="J27" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K27" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G27" s="36">
+      <c r="L27" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M27" s="23">
         <v>16.0</v>
       </c>
-      <c r="H27" s="37">
+      <c r="N27" s="24">
         <v>0.6388888888888888</v>
       </c>
-      <c r="I27" s="38" t="s">
+      <c r="O27" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="J27" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K27" s="38" t="s">
+      <c r="P27" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q27" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="L27" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M27" s="36">
+      <c r="R27" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="S27" s="44">
         <v>16.0</v>
       </c>
-      <c r="N27" s="37">
+      <c r="T27" s="60">
         <v>0.6388888888888888</v>
       </c>
-      <c r="O27" s="38" t="s">
+      <c r="U27" s="44"/>
+      <c r="V27" s="44"/>
+      <c r="W27" s="44"/>
+      <c r="X27" s="61"/>
+      <c r="Y27" s="57">
+        <v>16.0</v>
+      </c>
+      <c r="Z27" s="58">
+        <v>0.6388888888888888</v>
+      </c>
+      <c r="AA27" s="53" t="s">
         <v>55</v>
       </c>
-      <c r="P27" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q27" s="38" t="s">
+      <c r="AB27" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC27" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="R27" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S27" s="55">
-        <v>16.0</v>
-      </c>
-      <c r="T27" s="56">
-        <v>0.6388888888888888</v>
-      </c>
-      <c r="U27" s="55"/>
-      <c r="V27" s="55"/>
-      <c r="W27" s="55"/>
-      <c r="X27" s="57"/>
-      <c r="Y27" s="36">
-        <v>16.0</v>
-      </c>
-      <c r="Z27" s="37">
-        <v>0.6388888888888888</v>
-      </c>
-      <c r="AA27" s="38" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB27" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC27" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="AD27" s="38" t="s">
+      <c r="AD27" s="53" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="36">
+      <c r="A28" s="57">
         <v>17.0</v>
       </c>
-      <c r="B28" s="37">
+      <c r="B28" s="58">
         <v>0.6527777777777778</v>
       </c>
-      <c r="C28" s="58" t="s">
+      <c r="C28" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="57">
+        <v>17.0</v>
+      </c>
+      <c r="H28" s="58">
+        <v>0.6527777777777778</v>
+      </c>
+      <c r="I28" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E28" s="38" t="s">
+      <c r="J28" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="F28" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" s="36">
+      <c r="L28" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M28" s="57">
         <v>17.0</v>
       </c>
-      <c r="H28" s="37">
+      <c r="N28" s="58">
         <v>0.6527777777777778</v>
       </c>
-      <c r="I28" s="38" t="s">
+      <c r="O28" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="J28" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="K28" s="38" t="s">
+      <c r="P28" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q28" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="L28" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M28" s="36">
+      <c r="R28" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="S28" s="38">
         <v>17.0</v>
       </c>
-      <c r="N28" s="37">
+      <c r="T28" s="39">
         <v>0.6527777777777778</v>
       </c>
-      <c r="O28" s="38" t="s">
+      <c r="U28" s="38"/>
+      <c r="V28" s="38"/>
+      <c r="W28" s="38"/>
+      <c r="X28" s="38"/>
+      <c r="Y28" s="57">
+        <v>17.0</v>
+      </c>
+      <c r="Z28" s="58">
+        <v>0.6527777777777778</v>
+      </c>
+      <c r="AA28" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="P28" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q28" s="38" t="s">
+      <c r="AB28" s="63" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC28" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="R28" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S28" s="39">
-        <v>17.0</v>
-      </c>
-      <c r="T28" s="40">
-        <v>0.6527777777777778</v>
-      </c>
-      <c r="U28" s="39"/>
-      <c r="V28" s="39"/>
-      <c r="W28" s="39"/>
-      <c r="X28" s="39"/>
-      <c r="Y28" s="36">
-        <v>17.0</v>
-      </c>
-      <c r="Z28" s="37">
-        <v>0.6527777777777778</v>
-      </c>
-      <c r="AA28" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB28" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC28" s="45" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD28" s="59" t="s">
+      <c r="AD28" s="64" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="36">
+      <c r="A29" s="57">
         <v>18.0</v>
       </c>
-      <c r="B29" s="37">
+      <c r="B29" s="58">
         <v>0.6666666666666666</v>
       </c>
-      <c r="C29" s="38" t="s">
+      <c r="C29" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29" s="57">
+        <v>18.0</v>
+      </c>
+      <c r="H29" s="58">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="I29" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="D29" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E29" s="38" t="s">
+      <c r="J29" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K29" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="F29" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G29" s="36">
+      <c r="L29" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M29" s="57">
         <v>18.0</v>
       </c>
-      <c r="H29" s="37">
+      <c r="N29" s="58">
         <v>0.6666666666666666</v>
       </c>
-      <c r="I29" s="38" t="s">
+      <c r="O29" s="53" t="s">
         <v>62</v>
       </c>
-      <c r="J29" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K29" s="38" t="s">
+      <c r="P29" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q29" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="R29" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="S29" s="38">
+        <v>18.0</v>
+      </c>
+      <c r="T29" s="39">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="U29" s="38"/>
+      <c r="V29" s="38"/>
+      <c r="W29" s="38"/>
+      <c r="X29" s="38"/>
+      <c r="Y29" s="57">
+        <v>18.0</v>
+      </c>
+      <c r="Z29" s="58">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AA29" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="AB29" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC29" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="L29" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M29" s="36">
-        <v>18.0</v>
-      </c>
-      <c r="N29" s="37">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="O29" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="P29" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q29" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="R29" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="S29" s="39">
-        <v>18.0</v>
-      </c>
-      <c r="T29" s="40">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="U29" s="39"/>
-      <c r="V29" s="39"/>
-      <c r="W29" s="39"/>
-      <c r="X29" s="39"/>
-      <c r="Y29" s="36">
-        <v>18.0</v>
-      </c>
-      <c r="Z29" s="37">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AA29" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB29" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC29" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD29" s="38" t="s">
+      <c r="AD29" s="53" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="36">
+      <c r="A30" s="57">
         <v>19.0</v>
       </c>
-      <c r="B30" s="37">
+      <c r="B30" s="58">
         <v>0.6805555555555556</v>
       </c>
-      <c r="C30" s="38" t="s">
+      <c r="C30" s="53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30" s="57">
+        <v>19.0</v>
+      </c>
+      <c r="H30" s="58">
+        <v>0.6805555555555556</v>
+      </c>
+      <c r="I30" s="53" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E30" s="38" t="s">
+      <c r="J30" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K30" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="L30" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M30" s="57">
+        <v>19.0</v>
+      </c>
+      <c r="N30" s="58">
+        <v>0.6805555555555556</v>
+      </c>
+      <c r="O30" s="65" t="s">
+        <v>22</v>
+      </c>
+      <c r="P30" s="66" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q30" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="F30" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G30" s="36">
+      <c r="R30" s="66" t="s">
+        <v>16</v>
+      </c>
+      <c r="S30" s="63">
         <v>19.0</v>
       </c>
-      <c r="H30" s="37">
+      <c r="T30" s="67">
         <v>0.6805555555555556</v>
       </c>
-      <c r="I30" s="38" t="s">
+      <c r="U30" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="J30" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K30" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="L30" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M30" s="41">
+      <c r="V30" s="63" t="s">
+        <v>14</v>
+      </c>
+      <c r="W30" s="63" t="s">
+        <v>15</v>
+      </c>
+      <c r="X30" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y30" s="57">
         <v>19.0</v>
       </c>
-      <c r="N30" s="42">
+      <c r="Z30" s="58">
         <v>0.6805555555555556</v>
       </c>
-      <c r="O30" s="60" t="s">
+      <c r="AA30" s="53" t="s">
         <v>67</v>
       </c>
-      <c r="P30" s="61"/>
-      <c r="Q30" s="61"/>
-      <c r="R30" s="62"/>
-      <c r="S30" s="45">
-        <v>19.0</v>
-      </c>
-      <c r="T30" s="46">
-        <v>0.6805555555555556</v>
-      </c>
-      <c r="U30" s="45" t="s">
-        <v>68</v>
-      </c>
-      <c r="V30" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="W30" s="45" t="s">
+      <c r="AB30" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC30" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="X30" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y30" s="36">
-        <v>19.0</v>
-      </c>
-      <c r="Z30" s="37">
-        <v>0.6805555555555556</v>
-      </c>
-      <c r="AA30" s="38" t="s">
-        <v>69</v>
-      </c>
-      <c r="AB30" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC30" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD30" s="38" t="s">
+      <c r="AD30" s="53" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="36">
+      <c r="A31" s="57">
         <v>20.0</v>
       </c>
-      <c r="B31" s="37">
+      <c r="B31" s="58">
         <v>0.6944444444444444</v>
       </c>
-      <c r="C31" s="38" t="s">
+      <c r="C31" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="57">
+        <v>20.0</v>
+      </c>
+      <c r="H31" s="58">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="I31" s="53" t="s">
+        <v>69</v>
+      </c>
+      <c r="J31" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K31" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="L31" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M31" s="57">
+        <v>20.0</v>
+      </c>
+      <c r="N31" s="58">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="O31" s="59" t="s">
+        <v>28</v>
+      </c>
+      <c r="P31" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q31" s="53" t="s">
+        <v>27</v>
+      </c>
+      <c r="R31" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="S31" s="38">
+        <v>20.0</v>
+      </c>
+      <c r="T31" s="39">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="U31" s="38"/>
+      <c r="V31" s="38"/>
+      <c r="W31" s="38"/>
+      <c r="X31" s="38"/>
+      <c r="Y31" s="57">
+        <v>20.0</v>
+      </c>
+      <c r="Z31" s="58">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="AA31" s="53" t="s">
         <v>70</v>
       </c>
-      <c r="D31" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="F31" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G31" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="H31" s="37">
-        <v>0.6944444444444444</v>
-      </c>
-      <c r="I31" s="38" t="s">
-        <v>71</v>
-      </c>
-      <c r="J31" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K31" s="38" t="s">
+      <c r="AB31" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC31" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="L31" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M31" s="41">
-        <v>20.0</v>
-      </c>
-      <c r="N31" s="42">
-        <v>0.6944444444444444</v>
-      </c>
-      <c r="O31" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P31" s="61"/>
-      <c r="Q31" s="61"/>
-      <c r="R31" s="62"/>
-      <c r="S31" s="39">
-        <v>20.0</v>
-      </c>
-      <c r="T31" s="40">
-        <v>0.6944444444444444</v>
-      </c>
-      <c r="U31" s="39"/>
-      <c r="V31" s="39"/>
-      <c r="W31" s="39"/>
-      <c r="X31" s="39"/>
-      <c r="Y31" s="36">
-        <v>20.0</v>
-      </c>
-      <c r="Z31" s="37">
-        <v>0.6944444444444444</v>
-      </c>
-      <c r="AA31" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="AB31" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC31" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="AD31" s="38" t="s">
+      <c r="AD31" s="53" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="36">
+      <c r="A32" s="57">
         <v>21.0</v>
       </c>
-      <c r="B32" s="37">
+      <c r="B32" s="58">
         <v>0.7083333333333334</v>
       </c>
-      <c r="C32" s="38" t="s">
+      <c r="C32" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="57">
+        <v>21.0</v>
+      </c>
+      <c r="H32" s="58">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="I32" s="63" t="s">
+        <v>72</v>
+      </c>
+      <c r="J32" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="K32" s="63" t="s">
+        <v>15</v>
+      </c>
+      <c r="L32" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="M32" s="38">
+        <v>21.0</v>
+      </c>
+      <c r="N32" s="39">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="O32" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E32" s="38" t="s">
+      <c r="P32" s="70"/>
+      <c r="Q32" s="70"/>
+      <c r="R32" s="71"/>
+      <c r="S32" s="57">
+        <v>21.0</v>
+      </c>
+      <c r="T32" s="58">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="U32" s="72" t="s">
+        <v>74</v>
+      </c>
+      <c r="V32" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="W32" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="F32" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G32" s="36">
+      <c r="X32" s="72" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y32" s="57">
         <v>21.0</v>
       </c>
-      <c r="H32" s="37">
+      <c r="Z32" s="58">
         <v>0.7083333333333334</v>
       </c>
-      <c r="I32" s="63" t="s">
-        <v>74</v>
-      </c>
-      <c r="J32" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K32" s="38" t="s">
+      <c r="AA32" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB32" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC32" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="L32" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M32" s="41">
-        <v>21.0</v>
-      </c>
-      <c r="N32" s="42">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="O32" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P32" s="61"/>
-      <c r="Q32" s="61"/>
-      <c r="R32" s="62"/>
-      <c r="S32" s="36">
-        <v>21.0</v>
-      </c>
-      <c r="T32" s="37">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="U32" s="64" t="s">
-        <v>75</v>
-      </c>
-      <c r="V32" s="64" t="s">
-        <v>25</v>
-      </c>
-      <c r="W32" s="64" t="s">
-        <v>15</v>
-      </c>
-      <c r="X32" s="64" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y32" s="21">
-        <v>21.0</v>
-      </c>
-      <c r="Z32" s="22">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AA32" s="21"/>
-      <c r="AB32" s="21"/>
-      <c r="AC32" s="21"/>
-      <c r="AD32" s="21"/>
+      <c r="AD32" s="53" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="36">
+      <c r="A33" s="57">
         <v>22.0</v>
       </c>
-      <c r="B33" s="37">
+      <c r="B33" s="58">
         <v>0.7222222222222222</v>
       </c>
-      <c r="C33" s="38" t="s">
-        <v>76</v>
-      </c>
-      <c r="D33" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="E33" s="38" t="s">
+      <c r="C33" s="53" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G33" s="21">
+      <c r="F33" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33" s="57">
         <v>22.0</v>
       </c>
-      <c r="H33" s="22">
+      <c r="H33" s="58">
         <v>0.7222222222222222</v>
       </c>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="21"/>
-      <c r="M33" s="41">
+      <c r="I33" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="J33" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K33" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="L33" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M33" s="35">
         <v>22.0</v>
       </c>
-      <c r="N33" s="42">
+      <c r="N33" s="36">
         <v>0.7222222222222222</v>
       </c>
-      <c r="O33" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P33" s="61"/>
-      <c r="Q33" s="61"/>
-      <c r="R33" s="62"/>
-      <c r="S33" s="21">
+      <c r="O33" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P33" s="70"/>
+      <c r="Q33" s="70"/>
+      <c r="R33" s="71"/>
+      <c r="S33" s="57">
         <v>22.0</v>
       </c>
-      <c r="T33" s="22">
+      <c r="T33" s="58">
         <v>0.7222222222222222</v>
       </c>
-      <c r="U33" s="21"/>
-      <c r="V33" s="21"/>
-      <c r="W33" s="21"/>
-      <c r="X33" s="21"/>
+      <c r="U33" s="53" t="s">
+        <v>37</v>
+      </c>
+      <c r="V33" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="W33" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="X33" s="53" t="s">
+        <v>16</v>
+      </c>
       <c r="Y33" s="21">
         <v>22.0</v>
       </c>
@@ -3002,29 +3057,29 @@
         <v>0.7222222222222222</v>
       </c>
       <c r="AA33" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB33" s="21"/>
       <c r="AC33" s="21"/>
       <c r="AD33" s="21"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="36">
+      <c r="A34" s="57">
         <v>23.0</v>
       </c>
-      <c r="B34" s="37">
+      <c r="B34" s="58">
         <v>0.7361111111111112</v>
       </c>
-      <c r="C34" s="38" t="s">
+      <c r="C34" s="53" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="E34" s="38" t="s">
+      <c r="E34" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="F34" s="38" t="s">
+      <c r="F34" s="53" t="s">
         <v>16</v>
       </c>
       <c r="G34" s="21">
@@ -3037,18 +3092,18 @@
       <c r="J34" s="21"/>
       <c r="K34" s="21"/>
       <c r="L34" s="21"/>
-      <c r="M34" s="41">
+      <c r="M34" s="35">
         <v>23.0</v>
       </c>
-      <c r="N34" s="42">
+      <c r="N34" s="36">
         <v>0.7361111111111112</v>
       </c>
-      <c r="O34" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P34" s="61"/>
-      <c r="Q34" s="61"/>
-      <c r="R34" s="62"/>
+      <c r="O34" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P34" s="70"/>
+      <c r="Q34" s="70"/>
+      <c r="R34" s="71"/>
       <c r="S34" s="21">
         <v>23.0</v>
       </c>
@@ -3077,10 +3132,10 @@
       <c r="B35" s="22">
         <v>0.75</v>
       </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
       <c r="G35" s="21">
         <v>24.0</v>
       </c>
@@ -3091,18 +3146,18 @@
       <c r="J35" s="21"/>
       <c r="K35" s="21"/>
       <c r="L35" s="21"/>
-      <c r="M35" s="41">
+      <c r="M35" s="35">
         <v>24.0</v>
       </c>
-      <c r="N35" s="42">
+      <c r="N35" s="36">
         <v>0.75</v>
       </c>
-      <c r="O35" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P35" s="61"/>
-      <c r="Q35" s="61"/>
-      <c r="R35" s="62"/>
+      <c r="O35" s="74" t="s">
+        <v>79</v>
+      </c>
+      <c r="P35" s="70"/>
+      <c r="Q35" s="70"/>
+      <c r="R35" s="71"/>
       <c r="S35" s="21">
         <v>24.0</v>
       </c>
@@ -3125,16 +3180,24 @@
       <c r="AD35" s="21"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="21">
+      <c r="A36" s="57">
         <v>25.0</v>
       </c>
-      <c r="B36" s="22">
+      <c r="B36" s="58">
         <v>0.7638888888888888</v>
       </c>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
+      <c r="C36" s="53" t="s">
+        <v>29</v>
+      </c>
+      <c r="D36" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" s="53" t="s">
+        <v>16</v>
+      </c>
       <c r="G36" s="21">
         <v>25.0</v>
       </c>
@@ -3145,18 +3208,18 @@
       <c r="J36" s="21"/>
       <c r="K36" s="21"/>
       <c r="L36" s="21"/>
-      <c r="M36" s="41">
+      <c r="M36" s="35">
         <v>25.0</v>
       </c>
-      <c r="N36" s="42">
+      <c r="N36" s="36">
         <v>0.7638888888888888</v>
       </c>
-      <c r="O36" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P36" s="61"/>
-      <c r="Q36" s="61"/>
-      <c r="R36" s="62"/>
+      <c r="O36" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P36" s="70"/>
+      <c r="Q36" s="70"/>
+      <c r="R36" s="71"/>
       <c r="S36" s="21">
         <v>25.0</v>
       </c>
@@ -3189,36 +3252,36 @@
       <c r="D37" s="21"/>
       <c r="E37" s="21"/>
       <c r="F37" s="21"/>
-      <c r="G37" s="36">
+      <c r="G37" s="57">
         <v>26.0</v>
       </c>
-      <c r="H37" s="37">
+      <c r="H37" s="58">
         <v>0.7777777777777778</v>
       </c>
-      <c r="I37" s="38" t="s">
+      <c r="I37" s="53" t="s">
         <v>80</v>
       </c>
-      <c r="J37" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="K37" s="38" t="s">
+      <c r="J37" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="K37" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="L37" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="M37" s="41">
+      <c r="L37" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="M37" s="35">
         <v>26.0</v>
       </c>
-      <c r="N37" s="42">
+      <c r="N37" s="36">
         <v>0.7777777777777778</v>
       </c>
-      <c r="O37" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P37" s="61"/>
-      <c r="Q37" s="61"/>
-      <c r="R37" s="62"/>
+      <c r="O37" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P37" s="70"/>
+      <c r="Q37" s="70"/>
+      <c r="R37" s="71"/>
       <c r="S37" s="21">
         <v>26.0</v>
       </c>
@@ -3261,18 +3324,18 @@
       <c r="J38" s="21"/>
       <c r="K38" s="21"/>
       <c r="L38" s="21"/>
-      <c r="M38" s="41">
+      <c r="M38" s="35">
         <v>27.0</v>
       </c>
-      <c r="N38" s="42">
+      <c r="N38" s="36">
         <v>0.7916666666666666</v>
       </c>
-      <c r="O38" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P38" s="61"/>
-      <c r="Q38" s="61"/>
-      <c r="R38" s="62"/>
+      <c r="O38" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P38" s="70"/>
+      <c r="Q38" s="70"/>
+      <c r="R38" s="71"/>
       <c r="S38" s="21">
         <v>27.0</v>
       </c>
@@ -3315,18 +3378,18 @@
       <c r="J39" s="21"/>
       <c r="K39" s="21"/>
       <c r="L39" s="21"/>
-      <c r="M39" s="41">
+      <c r="M39" s="35">
         <v>28.0</v>
       </c>
-      <c r="N39" s="42">
+      <c r="N39" s="36">
         <v>0.8055555555555556</v>
       </c>
-      <c r="O39" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P39" s="61"/>
-      <c r="Q39" s="61"/>
-      <c r="R39" s="62"/>
+      <c r="O39" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P39" s="70"/>
+      <c r="Q39" s="70"/>
+      <c r="R39" s="71"/>
       <c r="S39" s="21">
         <v>28.0</v>
       </c>
@@ -3346,7 +3409,7 @@
       <c r="AA39" s="21"/>
       <c r="AB39" s="21"/>
       <c r="AC39" s="21"/>
-      <c r="AD39" s="65"/>
+      <c r="AD39" s="75"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="21">
@@ -3369,18 +3432,18 @@
       <c r="J40" s="21"/>
       <c r="K40" s="21"/>
       <c r="L40" s="21"/>
-      <c r="M40" s="41">
+      <c r="M40" s="35">
         <v>29.0</v>
       </c>
-      <c r="N40" s="42">
+      <c r="N40" s="36">
         <v>0.8194444444444444</v>
       </c>
-      <c r="O40" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P40" s="61"/>
-      <c r="Q40" s="61"/>
-      <c r="R40" s="62"/>
+      <c r="O40" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P40" s="70"/>
+      <c r="Q40" s="70"/>
+      <c r="R40" s="71"/>
       <c r="S40" s="21">
         <v>29.0</v>
       </c>
@@ -3400,7 +3463,7 @@
       <c r="AA40" s="21"/>
       <c r="AB40" s="21"/>
       <c r="AC40" s="21"/>
-      <c r="AD40" s="65"/>
+      <c r="AD40" s="75"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="21">
@@ -3423,18 +3486,18 @@
       <c r="J41" s="21"/>
       <c r="K41" s="21"/>
       <c r="L41" s="21"/>
-      <c r="M41" s="41">
+      <c r="M41" s="35">
         <v>30.0</v>
       </c>
-      <c r="N41" s="42">
+      <c r="N41" s="36">
         <v>0.8333333333333334</v>
       </c>
-      <c r="O41" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P41" s="61"/>
-      <c r="Q41" s="61"/>
-      <c r="R41" s="62"/>
+      <c r="O41" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P41" s="70"/>
+      <c r="Q41" s="70"/>
+      <c r="R41" s="71"/>
       <c r="S41" s="21">
         <v>30.0</v>
       </c>
@@ -3454,7 +3517,7 @@
       <c r="AA41" s="21"/>
       <c r="AB41" s="21"/>
       <c r="AC41" s="21"/>
-      <c r="AD41" s="65"/>
+      <c r="AD41" s="75"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="21">
@@ -3477,18 +3540,18 @@
       <c r="J42" s="21"/>
       <c r="K42" s="21"/>
       <c r="L42" s="21"/>
-      <c r="M42" s="41">
+      <c r="M42" s="35">
         <v>31.0</v>
       </c>
-      <c r="N42" s="42">
+      <c r="N42" s="36">
         <v>0.8472222222222222</v>
       </c>
-      <c r="O42" s="60" t="s">
-        <v>67</v>
-      </c>
-      <c r="P42" s="61"/>
-      <c r="Q42" s="61"/>
-      <c r="R42" s="62"/>
+      <c r="O42" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="P42" s="70"/>
+      <c r="Q42" s="70"/>
+      <c r="R42" s="71"/>
       <c r="S42" s="21">
         <v>31.0</v>
       </c>
@@ -3508,61 +3571,61 @@
       <c r="AA42" s="21"/>
       <c r="AB42" s="21"/>
       <c r="AC42" s="21"/>
-      <c r="AD42" s="65"/>
+      <c r="AD42" s="75"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="66">
+      <c r="A43" s="76">
         <v>32.0</v>
       </c>
-      <c r="B43" s="67">
+      <c r="B43" s="77">
         <v>0.8611111111111112</v>
       </c>
-      <c r="C43" s="66"/>
-      <c r="D43" s="66"/>
-      <c r="E43" s="66"/>
-      <c r="F43" s="66"/>
-      <c r="G43" s="66">
+      <c r="C43" s="76"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76">
         <v>32.0</v>
       </c>
-      <c r="H43" s="67">
+      <c r="H43" s="77">
         <v>0.8611111111111112</v>
       </c>
-      <c r="I43" s="66"/>
-      <c r="J43" s="66"/>
-      <c r="K43" s="66"/>
-      <c r="L43" s="66"/>
-      <c r="M43" s="68">
+      <c r="I43" s="76"/>
+      <c r="J43" s="76"/>
+      <c r="K43" s="76"/>
+      <c r="L43" s="76"/>
+      <c r="M43" s="78">
         <v>32.0</v>
       </c>
-      <c r="N43" s="69">
+      <c r="N43" s="79">
         <v>0.8611111111111112</v>
       </c>
-      <c r="O43" s="70" t="s">
-        <v>67</v>
-      </c>
-      <c r="P43" s="71"/>
-      <c r="Q43" s="71"/>
-      <c r="R43" s="72"/>
-      <c r="S43" s="66">
+      <c r="O43" s="80" t="s">
+        <v>73</v>
+      </c>
+      <c r="P43" s="81"/>
+      <c r="Q43" s="81"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="76">
         <v>32.0</v>
       </c>
-      <c r="T43" s="67">
+      <c r="T43" s="77">
         <v>0.8611111111111112</v>
       </c>
-      <c r="U43" s="66"/>
-      <c r="V43" s="66"/>
-      <c r="W43" s="66"/>
-      <c r="X43" s="66"/>
-      <c r="Y43" s="66">
+      <c r="U43" s="76"/>
+      <c r="V43" s="76"/>
+      <c r="W43" s="76"/>
+      <c r="X43" s="76"/>
+      <c r="Y43" s="76">
         <v>32.0</v>
       </c>
-      <c r="Z43" s="67">
+      <c r="Z43" s="77">
         <v>0.8611111111111112</v>
       </c>
-      <c r="AA43" s="66"/>
-      <c r="AB43" s="66"/>
-      <c r="AC43" s="66"/>
-      <c r="AD43" s="73"/>
+      <c r="AA43" s="76"/>
+      <c r="AB43" s="76"/>
+      <c r="AC43" s="76"/>
+      <c r="AD43" s="83"/>
     </row>
     <row r="44" ht="15.75" customHeight="1"/>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -4522,7 +4585,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="55">
+  <mergeCells count="53">
     <mergeCell ref="V10:V11"/>
     <mergeCell ref="W10:W11"/>
     <mergeCell ref="X10:X11"/>
@@ -4571,8 +4634,6 @@
     <mergeCell ref="O41:R41"/>
     <mergeCell ref="O42:R42"/>
     <mergeCell ref="O43:R43"/>
-    <mergeCell ref="O30:R30"/>
-    <mergeCell ref="O31:R31"/>
     <mergeCell ref="O32:R32"/>
     <mergeCell ref="O33:R33"/>
     <mergeCell ref="O34:R34"/>

</xml_diff>